<commit_message>
updated till mandatory questions & db fix
</commit_message>
<xml_diff>
--- a/SOW_Automation/Templates/Excel_Template.xlsx
+++ b/SOW_Automation/Templates/Excel_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\SOWautomation\SOW_Automation\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003904BE-A739-4AF4-8300-49154B708C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B3358B-1F08-4E23-A2F1-1FA16A3680EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B035CEB9-D536-4B4E-883F-C55C1F3FCF2A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary master" sheetId="1" r:id="rId1"/>
@@ -22,28 +22,12 @@
     <definedName name="_Ref507679024" localSheetId="0">'Summary master'!$D$24</definedName>
     <definedName name="_Ref508791623" localSheetId="0">'Summary master'!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="301">
   <si>
     <t>#</t>
   </si>
@@ -66,67 +50,122 @@
     <t>Automation steps</t>
   </si>
   <si>
+    <t>Variables</t>
+  </si>
+  <si>
+    <t>Parent</t>
+  </si>
+  <si>
+    <t>Mandatory</t>
+  </si>
+  <si>
     <t>XX Month 20XX</t>
   </si>
   <si>
+    <t>Please fill as per Summary Text</t>
+  </si>
+  <si>
+    <t>SOW_DATE</t>
+  </si>
+  <si>
     <t>INSERT EY FIRM LEGAL NAME</t>
   </si>
   <si>
+    <t>FIRM_LEGAL_NAME</t>
+  </si>
+  <si>
     <t>INSERT CLIENT FULL LEGAL NAME</t>
   </si>
   <si>
+    <t>CLIENT_FULL_LEGAL_NAME</t>
+  </si>
+  <si>
     <t>on behalf of itself and its affiliated entities listed in Schedule 1 of the Cover Letter</t>
   </si>
   <si>
+    <t>Please select 'No' if not applicable</t>
+  </si>
+  <si>
     <t>INSERT ABBREVIATED CLIENT NAME</t>
   </si>
   <si>
+    <t>ABV_CLIENT_NAME</t>
+  </si>
+  <si>
     <t xml:space="preserve">INSERT DATE OF COVER LETTER </t>
   </si>
   <si>
+    <t>COVER_LETTER_DATE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Effective Date” the date the Parties sign (binding contract); </t>
   </si>
   <si>
     <t>Effective Date” - Contract signing date</t>
   </si>
   <si>
+    <t>EFFECTIVE_DATE</t>
+  </si>
+  <si>
     <t xml:space="preserve">“Commencement Date” the date the Onboarding (or Transfer) Services Start; </t>
   </si>
   <si>
     <t>“Commencement Date” the date the Onboarding / transition starts</t>
   </si>
   <si>
+    <t>COMMENCEMENT_DATE</t>
+  </si>
+  <si>
     <t>“Go-Live Date” when the Managed Services Start (may be more than one Go-Live Date (e.g., for phased start of services)</t>
   </si>
   <si>
     <t>“Go-Live Date” when the Managed Services Start (may be more than one Go-Live Date e.g., for phased start of services)</t>
   </si>
   <si>
+    <t>GO_LIVE_DATE</t>
+  </si>
+  <si>
     <t xml:space="preserve">insert meaningful, yet high level summary of the services, e.g. “regulatory reporting” or “anti-money laundering monitoring” or “fraud detection” </t>
   </si>
   <si>
     <t xml:space="preserve">High level 2/3 word summary of the services, e.g. “regulatory reporting” or “anti-money laundering monitoring” or “fraud detection” </t>
   </si>
   <si>
+    <t>Please fill as per Summary Text, Maximum of 2 to 3 words</t>
+  </si>
+  <si>
     <t>NOTE TO DRAFT: Summarize the Scope of Services that will be described in Schedule A.  Note, consult with applicable subject matter resources to the extent the scope will involve the transition of client personnel (e.g., to EY), transfer of assets or the transfer or transformation of services (i.e., EY inheriting, then changing a service</t>
   </si>
   <si>
     <t xml:space="preserve"> Summarize the Scope of Services,  described in Schedule A</t>
   </si>
   <si>
+    <t>Please fill as per Summary Text, Maximum of 2 to 3 lines</t>
+  </si>
+  <si>
     <t>1a</t>
   </si>
   <si>
+    <t>a.	“Onboarding Services” – Starting on the Commencement Date, EY will work with Client to perform [describe …] to enable the Managed Services.</t>
+  </si>
+  <si>
     <t>Summary of the one-time, onboarding / transitioning scope at the start of the project</t>
   </si>
   <si>
-    <t>a.	“Onboarding Services” – Starting on the Commencement Date, EY will work with Client to perform [describe …] to enable the Managed Services.</t>
+    <t>ONBOARDING_SVC_DESCRIPTION</t>
   </si>
   <si>
     <t>1b</t>
   </si>
   <si>
+    <t xml:space="preserve">Starting on the Go-Live Date, EY will work the Client to perform [describe …].  The Parties anticipate that the “Go-Live Date” for the Managed Services will be:  **.GO_LIVE_DATE**.
+[NOTE TO DRAFT: Provide brief summary of the managed services, which are the ongoing services we perform for the term of the Agreement.  The details will be in Schedule A (Description of Services).]  </t>
+  </si>
+  <si>
     <t>Summary of the ongoing services  for the term of the Agreement</t>
+  </si>
+  <si>
+    <t>MANAGED_SVC_DESCRIPTION</t>
   </si>
   <si>
     <t>1c</t>
@@ -140,6 +179,12 @@
 regulatory mandates and/or - Update as required</t>
   </si>
   <si>
+    <t>Please mention 'NA' if not applicable, otherwise Please fill as per Summary Text</t>
+  </si>
+  <si>
+    <t>_ADD1, ADDITIONAL_SVC, _ADD2</t>
+  </si>
+  <si>
     <t>following assumptions, the following client responsibilities and other express</t>
   </si>
   <si>
@@ -148,6 +193,9 @@
 Option 2 - assumptions</t>
   </si>
   <si>
+    <t>Please select one option from Summary Text</t>
+  </si>
+  <si>
     <t>6a</t>
   </si>
   <si>
@@ -158,7 +206,13 @@
 EY will provides guidance, not decisions, on client accounting policy choices.</t>
   </si>
   <si>
+    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text</t>
+  </si>
+  <si>
     <t>6b</t>
+  </si>
+  <si>
+    <t>b.	[NOTE TO DRAFT: Include language in brackets if financial accounting and reporting services will be provided] The Services support Client’s business operations and are advisory in nature. EY will not render an assurance report or opinion under this SOW, nor will the Services constitute an audit, review, examination, or other form of assurance as those terms are defined by [Insert the International Auditing and Assurance Standards Board (IAASB) or relevant local standards]. *[Accordingly, EY will not express any form of assurance on accounting matters, financial statements, any financial or other information or internal controls as part of the Services.]* None of the Services or any reports will constitute any legal opinion or advice. EY will not conduct a review to detect fraud or illegal acts.</t>
   </si>
   <si>
     <t>MS scope - financial accounting and reporting services
@@ -176,50 +230,47 @@
 if appropriate, insert  relevant local standards</t>
   </si>
   <si>
+    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text
+Please update 3rd point, if applicable</t>
+  </si>
+  <si>
     <t>6k</t>
   </si>
   <si>
     <t>k.	[NOTE TO DRAFT: Add if Functional Deliverables are expressly anticipated in Schedule A (Description of Services)]  Without limitation to the provisions of Section 5 of the General Terms and Conditions of the Agreement, EY warrants that the Functional Deliverables will materially conform with their applicable specifications as may be described in Schedule A (Description of Services). If such Functional Deliverables do not materially conform to such specifications, and Client notifies EY of the nonconformity within [thirty (30)] days following delivery of the applicable Functional Deliverable, EY will correct such Functional Deliverable. EY’s obligation to correct such non-conforming Functional Deliverables will be Client’s sole remedy for breach of the warranty set forth in this Section 6.k. THE WARRANTY SET FORTH IN THIS SECTION 6.k IS IN LIEU OF ANY OTHER WARRANTIES BY EY, EXPRESS OR IMPLIED, ALL OF WHICH ARE HEREBY WAIVED BY CLIENT. [NOTE TO DRAFT: In the managed services context, Service performance is typically subject to Service Levels (see Schedule B) rather than a warranty.  This provision is added where there are Functional Deliverables either during the Onboarding phase or the managed service itself generates Functional Deliverables (e.g., a managed service that results in software deliverables).]</t>
   </si>
   <si>
-    <r>
-      <t>there are Functional Deliverables, e.g., software deliverables - workflow, interface, reports 
- If such Functional Deliverables do not materially conform to such specifications, and Client notifies EY of the nonconformity within</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> [thirty (30)] </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">days following delivery of the applicable Functional Deliverable, EY will correct such Functional Deliverable. </t>
-    </r>
+    <t xml:space="preserve">there are Functional Deliverables, e.g., software deliverables - workflow, interface, reports 
+ If such Functional Deliverables do not materially conform to such specifications, and Client notifies EY of the nonconformity within [thirty (30)] days following delivery of the applicable Functional Deliverable, EY will correct such Functional Deliverable. </t>
+  </si>
+  <si>
+    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
+Please update text in 2nd point, if applicable</t>
   </si>
   <si>
     <t>6l</t>
   </si>
   <si>
+    <t>l.	[NOTE TO DRAFT: Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO to modify the SOW template to conform with local requirements as needed.] [To the fullest extent permitted by applicable law and professional obligations, EY will indemnify Client against all liabilities, losses, damages, costs and expenses that are finally awarded by an arbitrator or court of competent jurisdiction, or included in a settlement pursuant to item (i) of this Section 6.l (below), due to third party claims alleging that the Services as performed by EY infringe a [insert jurisdiction in which the services are being provided]  patent, copyright, trade secret or other registered intellectual property rights, provided that Client: (i) promptly notifies EY of such a claim; (ii) allows EY to control the defense or settlement of such claim; and (iii) provides EY with reasonable assistance in defending such claim. EY’s indemnification obligations in this Section 6.l shall not be applicable to the extent Client modifies the Services or combines them with other items not provided by EY, Client’s noncompliance with EY’s specifications for the Services or the terms of this SOW, or where the claim resulted from Client’s direction or specification. In the event of such a claim (or where EY believes such a claim is reasonably likely to occur), EY may, at its option: (A) modify the Service to be non-infringing; (B) obtain the rights to the affected Service; (C) replace the affected Service with a functionally equivalent service or item that is not infringing; or (D) if none of the foregoing is reasonably available, require that Client cease using the affected Service and provide an equitable pro-rata refund, based on the benefit received by Client prior to the cessation of use.  EY’s obligations under this Section 6.l are Client’s sole remedy and EY’s exclusive obligation in the event of a third party claim alleging that the Services as performed by EY infringe applicable intellectual property rights.]</t>
+  </si>
+  <si>
     <t>EY indemnifies Client for third-party IP infringement claims on Services, subject to Client’s cooperation and exclusions; EY may modify, replace, or refund affected Services as sole remedy.</t>
   </si>
   <si>
+    <t xml:space="preserve">Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
+Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO, modify if required
+</t>
+  </si>
+  <si>
     <t>6m</t>
   </si>
   <si>
     <t>m.	Client will not, and will not permit others to, quote or refer to the Deliverables, Performance Reports or other Output of the Services, any portion, summary or abstract thereof, or to EY or any other EY Firm, in any document filed or distributed in connection with (i) a purchase or sale of securities to which [reference jurisdictional securities laws]  (“Securities Laws”) are applicable, or (ii) periodic reporting obligations under Securities Laws. Client will not contend that any provisions of Securities Laws could invalidate any provision of this SOW.</t>
   </si>
   <si>
+    <t>Please mention the applicable  jurisdictional securities laws, e.g., UAE security laws</t>
+  </si>
+  <si>
     <t>6n</t>
   </si>
   <si>
@@ -232,7 +283,13 @@
     <t>6o</t>
   </si>
   <si>
+    <t xml:space="preserve">o.	[NOTE TO DRAFT: Include if financial accounting and reporting services will be provided and the services will be subject to audit by the Client’s external auditor] [Client is responsible for obtaining the concurrence of its external auditor on the appropriateness of the accounting policies that Client has selected and the related financial statement disclosures. Consider adding: Client will arrange for periodic status meetings with its external auditor that include representatives from Client, EY, and [Insert legal name of the client’s external auditor]. Client also agrees that EY can discuss the nature of the Services and consult with **EXTERNAL_AUDITOR** throughout the engagement with a view of understanding their positions in relation with accounting, financial reporting matters applicable to Client. Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO whether local laws or regulations do require a more explicit waiver from confidentiality obligations for such discussions with the Client’s external auditor.] </t>
+  </si>
+  <si>
     <t>Scope - financial accounting and reporting services subject to audit by the Client’s external auditor</t>
+  </si>
+  <si>
+    <t>FIN_ACCOUNTING,[EXTERNAL_AUDITOR]</t>
   </si>
   <si>
     <t>6q</t>
@@ -258,6 +315,10 @@
   <si>
     <t>Scope - involves outbound email
  [Insert relevant/applicable laws (e.g., CAN-SPAM Act of 2003]</t>
+  </si>
+  <si>
+    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
+Please update red text in 2nd point, if applicable</t>
   </si>
   <si>
     <t>6t</t>
@@ -271,7 +332,13 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Summary Text - 1st point is mandatory, Please select 'Yes' or 'No' on the 2nd point </t>
+  </si>
+  <si>
     <t>6u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">u.	[Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO to modify this clause to conform with local requirements as needed. For purposes of this SOW, Client may not recover from EY, in contract or tort, under statute or otherwise, damages that exceed, in the aggregate for all claims arising out of this SOW, the fees paid by Client to EY for the Services during the {six (6) / twelve (12)}-month period immediately preceding the events giving rise to the most recent claim (“Direct Damages Cap”). *{}* [NOTE TO DRAFT:  Teams are advised to consider carefully the starting point for liability for Managed Services, which may vary by offering.  Also, consider carefully and client request for a “floor” or ramp-up process for liability, which may precede EY being paid fees by the Client..]  </t>
   </si>
   <si>
     <t>Client’s recoverable damages from EY are capped at fees paid in the prior 6–12 months for Services under this SOW.</t>
@@ -323,6 +390,13 @@
 the client asks that we leave behind any technology or EY Tools after the Term.  This case should be addressed as part of termination scenarios in Section 7</t>
   </si>
   <si>
+    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text
+Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO if 2nd point is applicable</t>
+  </si>
+  <si>
+    <t>CLIENT_ENV_TOOL</t>
+  </si>
+  <si>
     <t>6cc</t>
   </si>
   <si>
@@ -342,6 +416,9 @@
   </si>
   <si>
     <t>7a</t>
+  </si>
+  <si>
+    <t>The Services under this SOW shall begin as of **COMMENCEMENT_DATE** (the “Commencement Date”) and end on the date that is  [XX] months after the Go-Live Date (the “Term”).   [NOTE TO DRAFT:  A typical structure might provide for a defined number of months for the Managed Services in relation to the Go-Live Date (or the last of the Go-Live Dates if there is more than one), so that here is a single, coordinated end of the Term for the Managed Services.]</t>
   </si>
   <si>
     <t>Commencement Date
@@ -352,7 +429,13 @@
 Update XX</t>
   </si>
   <si>
+    <t>Please update commencement date from above</t>
+  </si>
+  <si>
     <t>7b</t>
+  </si>
+  <si>
+    <t>b.	Renewal.  No fewer than [x (x) ]months prior to the expiration of the Term of this SOW (or any renewal term), the Parties will enter into good faith negotiations with each other regarding the adjustment of any terms and conditions to this SOW, including the duration of renewal term, scope of services, and charges, which will be implemented in accordance with the Change Control Procedures.  Any agreed renewal term will extend the Term for an additional period of [x (x)] years, unless otherwise agreed to by the Parties in writing.  [NOTE TO DRAFT:  This is a mutual formulation of a renewal process, and recognizes that terms and pricing may need to be re-negotiated.  Consult with subject matter resources about other formulations (e.g., defined client option years).]</t>
   </si>
   <si>
     <t>Renewal negotiation x months prior to the expiration of the Term of this SOW
@@ -371,6 +454,10 @@
     <t xml:space="preserve">Client may elect to terminate this SOW (in whole, but not in part) prior to the end of the Term by giving EY at least [90] days written notice provided, however, that Client may not exercise such right prior to the date that is ## days after the Go-Live Date.  </t>
   </si>
   <si>
+    <t>Please update '90' days if required
+Please update ## if Applicable. If not, say 'NA'</t>
+  </si>
+  <si>
     <t>7c2</t>
   </si>
   <si>
@@ -380,146 +467,43 @@
     <t>Either Party may terminate this SOW, immediately, upon written notice if the other Party materially breaches this SOW and such breach is not cured within [60] days following receipt of the written notice</t>
   </si>
   <si>
+    <t>Please update '60' days if required</t>
+  </si>
+  <si>
     <t>8b</t>
   </si>
   <si>
+    <t>EY will make the Transfer Assistance Services available for up to [(x)] additional months after the effective date of expiration or termination.</t>
+  </si>
+  <si>
     <t xml:space="preserve">EY will make the Transfer Assistance Services available for up to (x) additional months after the effective date of expiration or termination. </t>
   </si>
   <si>
+    <t>Please update x</t>
+  </si>
+  <si>
     <t>[Service Levels will not apply during any period of Transfer Assistance Services after the effective date of expiration or termination.] [NOTE TO DRAFT: Typically 3-6 months.  Delete last sentence if Service Levels are not applicable.]</t>
   </si>
   <si>
     <t xml:space="preserve"> Service Levels are applicable</t>
   </si>
   <si>
+    <t>Please answer 'Yes' or 'No'</t>
+  </si>
+  <si>
     <t>9a</t>
   </si>
   <si>
+    <t>a.	Deliverables. [In connection with the Onboarding Services,] Following delivery of a Deliverable by EY, Client will conduct promptly the applicable acceptance test or review, and inform EY of Client’s acceptance or rejection of such Deliverable. Any rejection by Client must specify the material deficiencies of the Deliverable as compared to the applicable acceptance test criteria or applicable written requirements for the Deliverable. If Client fails to accept or reject such Deliverable within the period of time specified in Exhibit A, (or [2 business] days after delivery if not specified), the Deliverable will be deemed accepted.  If Client delivers to EY a timely notice of deficiencies and the items specified in the notice are deficiencies, EY will correct the described deficiencies within a reasonable period of time. [Fixed Price: EY’s correction efforts will be made at no additional charge.}  {T&amp;M: EY’s correction efforts will be made on a time and materials basis.]  Upon receipt of a corrected Deliverable from EY, Client will have a reasonable additional period of time, not to exceed [3 business] days, to review the corrected Deliverable to confirm that the identified and agreed-upon deficiencies have been corrected. Client will not unreasonably withhold, delay or condition its approval of a Deliverable.  [NOTE TO DRAFT:  Include Section 9.a generally.  If there will be Functional Deliverables provided to the client as part of the Services, include Section 9.b as well.  In addition, the Functional Deliverables acceptance language assumes a process where there will be regular formal acceptance test steps (generally UAT), and may need to be separately tailored for an Agile or DevOps approach to development.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If Client fails to accept or reject Deliverable within time specified in Exhibit A, (or {3 business} days after delivery if not specified), the Deliverable will be deemed accepted. Then select Fixed price or T&amp;M. Also clarify "Upon receipt of a corrected Deliverable from EY, Client will have an additional upto  {3 business} days, to review the corrected Deliverable".</t>
+  </si>
+  <si>
+    <t>**1 Please answer 'Yes' or 'No'.                   **1a If appropriate consider limiting Section 9.a to “In connection with the Onboarding Services,…” if all Deliverables will occur during the Onboarding phase.               **1b fill the number of days.           **1c  Option 1: Fixed Price: EY’s correction efforts will be made at no additional charge. Option 2:T&amp;M: EY’s correction efforts will be made on a time and materials basis.           **1d fill the number of days.</t>
+  </si>
+  <si>
     <t>9b</t>
-  </si>
-  <si>
-    <t>Functional Deliverables provided to the client as part of the Services
-acceptance period for Functional Deliverables will be {x} days</t>
-  </si>
-  <si>
-    <t>11a</t>
-  </si>
-  <si>
-    <t>Client single point of contact</t>
-  </si>
-  <si>
-    <t>11b</t>
-  </si>
-  <si>
-    <t>EY single point of contact</t>
-  </si>
-  <si>
-    <t>Onboarding Services - general high-level objective
-Onboarding Services - general high-level description of services</t>
-  </si>
-  <si>
-    <t>Sch A 3</t>
-  </si>
-  <si>
-    <t>[NOTE TO DRAFT: Use the following if the Services involve assisting the Client in drafting its conclusions, including its accounting policy manual, as appropriate.] EY will assist Client in documenting its conclusions reached or positions taken on accounting and reporting matters, including the accounting policies Client has selected.</t>
-  </si>
-  <si>
-    <t>Scope - drafting conclusions, including accounting policy manual</t>
-  </si>
-  <si>
-    <t>iii.	Secure Workplace [NOTE TO DRAFT:  Add if EY is providing services from secure bays, as they will drive EY costs.  Be clear where secure bays are being used and which services the secure bays support (to manage costs and scope).] 
-Services in [location(s)] will be conducted out of a Secure Workplace.  Service locations may not be changed without the express written consent of Client.</t>
-  </si>
-  <si>
-    <t>EY is providing services from secure bays, as they will drive EY costs
-location(s)</t>
-  </si>
-  <si>
-    <t>Sch A 5b1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">i.	Client shall provide the following environment(s): {Specify the development, testing, integration, implementation and other environments to be provided by Client}. </t>
-  </si>
-  <si>
-    <t>Scope - IT implementation / Operation
-Specify the development, testing, integration, implementation and other environments to be provided by Client</t>
-  </si>
-  <si>
-    <t>Sch A 5b6</t>
-  </si>
-  <si>
-    <t>Scope - IT implementation / Operation
-Implemented/Integrated Software</t>
-  </si>
-  <si>
-    <t>Sch A 5b7</t>
-  </si>
-  <si>
-    <t>Scope - IT implementation 
-Implemented/Software</t>
-  </si>
-  <si>
-    <t>If 'No', delete the entire schedule on Service Level Methodology, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>If 'No', delete the entire schedule on Governance and Change Control, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>Sch E</t>
-  </si>
-  <si>
-    <t>If 'No', delete the entire schedule on Access and Technology Requirements, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>If 'No', delete the entire schedule on Disaster Recovery Plan, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>Client-Environment EY Tool</t>
-  </si>
-  <si>
-    <t>DR Plan</t>
-  </si>
-  <si>
-    <t>Dispute</t>
-  </si>
-  <si>
-    <t>CLIENT AFFILIATES</t>
-  </si>
-  <si>
-    <t>Ref</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Affiliate Entity Name </t>
-  </si>
-  <si>
-    <t>Registered Address</t>
-  </si>
-  <si>
-    <t>INSERT FULL LEGAL FIRM NAME</t>
-  </si>
-  <si>
-    <t>OR INSERT as appliable</t>
-  </si>
-  <si>
-    <t>All yellow highlighted text needs to be either updated or deleted</t>
-  </si>
-  <si>
-    <t>All text enclosed in [ ] need to be either updated or deleted</t>
-  </si>
-  <si>
-    <t>All text enclosed in [ ] and starting with "NOTE TO DRAFT" need to be deleted</t>
-  </si>
-  <si>
-    <t>All text enclosed in [ ] and not starting with "NOTE TO DRAFT" need to be updated or deleted</t>
-  </si>
-  <si>
-    <t>All text highlighted in blue need not be touched unless specifically mentioned in the clause wise rules</t>
-  </si>
-  <si>
-    <t>b.	Renewal.  No fewer than [x (x) ]months prior to the expiration of the Term of this SOW (or any renewal term), the Parties will enter into good faith negotiations with each other regarding the adjustment of any terms and conditions to this SOW, including the duration of renewal term, scope of services, and charges, which will be implemented in accordance with the Change Control Procedures.  Any agreed renewal term will extend the Term for an additional period of [x (x)] years, unless otherwise agreed to by the Parties in writing.  [NOTE TO DRAFT:  This is a mutual formulation of a renewal process, and recognizes that terms and pricing may need to be re-negotiated.  Consult with subject matter resources about other formulations (e.g., defined client option years).]</t>
   </si>
   <si>
     <t>b.	Functional Deliverables.  Acceptance testing for Functional Deliverables is an iterative process designed to determine whether the Functional Deliverable performs the functions described in the [Approved Design].  For Functional Deliverables, Nonconformities are the “material deficiencies” that may be discovered and removed through repeated testing cycles.  The process described in Section 9.a will apply, subject to the following:
@@ -528,119 +512,406 @@
 iii.	If EY does not receive notice identifying a material Nonconformity from Client during acceptance period for Functional Deliverables or Client begins using the Functional Deliverable in a production environment, the Functional Deliverable shall be deemed to be accepted.</t>
   </si>
   <si>
-    <t>Variables</t>
-  </si>
-  <si>
-    <t>SOW_DATE</t>
-  </si>
-  <si>
-    <t>FIRM_LEGAL_NAME</t>
-  </si>
-  <si>
-    <t>CLIENT_FULL_LEGAL_NAME</t>
-  </si>
-  <si>
-    <t>ABV_CLIENT_NAME</t>
-  </si>
-  <si>
-    <t>COVER_LETTER_DATE</t>
-  </si>
-  <si>
-    <t>EFFECTIVE_DATE</t>
-  </si>
-  <si>
-    <t>COMMENCEMENT_DATE</t>
-  </si>
-  <si>
-    <t>GO_LIVE_DATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Starting on the Go-Live Date, EY will work the Client to perform [describe …].  The Parties anticipate that the “Go-Live Date” for the Managed Services will be:  **.GO_LIVE_DATE**.
-[NOTE TO DRAFT: Provide brief summary of the managed services, which are the ongoing services we perform for the term of the Agreement.  The details will be in Schedule A (Description of Services).]  </t>
-  </si>
-  <si>
-    <t>l.	[NOTE TO DRAFT: Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO to modify the SOW template to conform with local requirements as needed.] [To the fullest extent permitted by applicable law and professional obligations, EY will indemnify Client against all liabilities, losses, damages, costs and expenses that are finally awarded by an arbitrator or court of competent jurisdiction, or included in a settlement pursuant to item (i) of this Section 6.l (below), due to third party claims alleging that the Services as performed by EY infringe a [insert jurisdiction in which the services are being provided]  patent, copyright, trade secret or other registered intellectual property rights, provided that Client: (i) promptly notifies EY of such a claim; (ii) allows EY to control the defense or settlement of such claim; and (iii) provides EY with reasonable assistance in defending such claim. EY’s indemnification obligations in this Section 6.l shall not be applicable to the extent Client modifies the Services or combines them with other items not provided by EY, Client’s noncompliance with EY’s specifications for the Services or the terms of this SOW, or where the claim resulted from Client’s direction or specification. In the event of such a claim (or where EY believes such a claim is reasonably likely to occur), EY may, at its option: (A) modify the Service to be non-infringing; (B) obtain the rights to the affected Service; (C) replace the affected Service with a functionally equivalent service or item that is not infringing; or (D) if none of the foregoing is reasonably available, require that Client cease using the affected Service and provide an equitable pro-rata refund, based on the benefit received by Client prior to the cessation of use.  EY’s obligations under this Section 6.l are Client’s sole remedy and EY’s exclusive obligation in the event of a third party claim alleging that the Services as performed by EY infringe applicable intellectual property rights.]</t>
-  </si>
-  <si>
-    <t>FIN_ACCOUNTING,[EXTERNAL_AUDITOR]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">o.	[NOTE TO DRAFT: Include if financial accounting and reporting services will be provided and the services will be subject to audit by the Client’s external auditor] [Client is responsible for obtaining the concurrence of its external auditor on the appropriateness of the accounting policies that Client has selected and the related financial statement disclosures. Consider adding: Client will arrange for periodic status meetings with its external auditor that include representatives from Client, EY, and [Insert legal name of the client’s external auditor]. Client also agrees that EY can discuss the nature of the Services and consult with **EXTERNAL_AUDITOR** throughout the engagement with a view of understanding their positions in relation with accounting, financial reporting matters applicable to Client. Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO whether local laws or regulations do require a more explicit waiver from confidentiality obligations for such discussions with the Client’s external auditor.] </t>
-  </si>
-  <si>
-    <t xml:space="preserve">u.	[Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO to modify this clause to conform with local requirements as needed. For purposes of this SOW, Client may not recover from EY, in contract or tort, under statute or otherwise, damages that exceed, in the aggregate for all claims arising out of this SOW, the fees paid by Client to EY for the Services during the {six (6) / twelve (12)}-month period immediately preceding the events giving rise to the most recent claim (“Direct Damages Cap”). *{}* [NOTE TO DRAFT:  Teams are advised to consider carefully the starting point for liability for Managed Services, which may vary by offering.  Also, consider carefully and client request for a “floor” or ramp-up process for liability, which may precede EY being paid fees by the Client..]  </t>
-  </si>
-  <si>
-    <t>CLIENT_ENV_TOOL</t>
-  </si>
-  <si>
-    <t>**1 Please answer 'Yes' or 'No'.                   **1a If appropriate consider limiting Section 9.a to “In connection with the Onboarding Services,…” if all Deliverables will occur during the Onboarding phase.               **1b fill the number of days.           **1c  Option 1: Fixed Price: EY’s correction efforts will be made at no additional charge. Option 2:T&amp;M: EY’s correction efforts will be made on a time and materials basis.           **1d fill the number of days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> If Client fails to accept or reject Deliverable within time specified in Exhibit A, (or {3 business} days after delivery if not specified), the Deliverable will be deemed accepted. Then select Fixed price or T&amp;M. Also clarify "Upon receipt of a corrected Deliverable from EY, Client will have an additional upto  {3 business} days, to review the corrected Deliverable".</t>
+    <t>Functional Deliverables provided to the client as part of the Services
+acceptance period for Functional Deliverables will be {x} days</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No'
+If 'yes', Please update x</t>
+  </si>
+  <si>
+    <t>11a</t>
   </si>
   <si>
     <t xml:space="preserve">a.      Client has identified [___] as its contact with whom EY should communicate about the Services under this SOW. </t>
   </si>
   <si>
+    <t>Client single point of contact</t>
+  </si>
+  <si>
+    <t>Please provide the full name</t>
+  </si>
+  <si>
+    <t>11b</t>
+  </si>
+  <si>
     <t>b.      Client’s contact at EY for the Services under this SOW will be [____].</t>
   </si>
   <si>
-    <t>a.	Deliverables. [In connection with the Onboarding Services,] Following delivery of a Deliverable by EY, Client will conduct promptly the applicable acceptance test or review, and inform EY of Client’s acceptance or rejection of such Deliverable. Any rejection by Client must specify the material deficiencies of the Deliverable as compared to the applicable acceptance test criteria or applicable written requirements for the Deliverable. If Client fails to accept or reject such Deliverable within the period of time specified in Exhibit A, (or [2 business] days after delivery if not specified), the Deliverable will be deemed accepted.  If Client delivers to EY a timely notice of deficiencies and the items specified in the notice are deficiencies, EY will correct the described deficiencies within a reasonable period of time. [Fixed Price: EY’s correction efforts will be made at no additional charge.}  {T&amp;M: EY’s correction efforts will be made on a time and materials basis.]  Upon receipt of a corrected Deliverable from EY, Client will have a reasonable additional period of time, not to exceed [3 business] days, to review the corrected Deliverable to confirm that the identified and agreed-upon deficiencies have been corrected. Client will not unreasonably withhold, delay or condition its approval of a Deliverable.  [NOTE TO DRAFT:  Include Section 9.a generally.  If there will be Functional Deliverables provided to the client as part of the Services, include Section 9.b as well.  In addition, the Functional Deliverables acceptance language assumes a process where there will be regular formal acceptance test steps (generally UAT), and may need to be separately tailored for an Agile or DevOps approach to development.]</t>
+    <t>EY single point of contact</t>
+  </si>
+  <si>
+    <t>Sch_A</t>
+  </si>
+  <si>
+    <t>*****A_Schedule*****</t>
+  </si>
+  <si>
+    <t>Description of Services</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability</t>
+  </si>
+  <si>
+    <t>Sch A1bi</t>
+  </si>
+  <si>
+    <t>**ONBOARDING_SVC_DESCRIPTION** as described in Section 1.f</t>
+  </si>
+  <si>
+    <t>Sch A1bii</t>
+  </si>
+  <si>
+    <t>**MANAGED_SVC_DESCRIPTION** as described in Section 3</t>
+  </si>
+  <si>
+    <t>Sch A1biii</t>
+  </si>
+  <si>
+    <t>**ADDITIONAL_SVC** Services as described in Section 4</t>
   </si>
   <si>
     <t>Sch A 1f</t>
   </si>
   <si>
+    <t>f.	EY will conduct the Services under this SOW pursuant to Client’s documented policies and procedures (“Client **CLIENT_FULL_LEGAL_NAME** Procedures”), which as of the Go Live Date is “[Insert Name of Procedures]”, dated **GO_LIVE_DATE** .   Any changes in Client **CLIENT_FULL_LEGAL_NAME** Procedures requested or initiated by Client during the Term will be implemented in accordance with the Change Control Procedures.</t>
+  </si>
+  <si>
+    <t>Sch A 2ai</t>
+  </si>
+  <si>
+    <t>[and after Client has completed the necessary technology development activities as described in Schedule E (Access and Technology Requirements)],</t>
+  </si>
+  <si>
+    <t>Beginning on the Commencement Date [and after Client has completed the necessary technology development activities as described in Schedule E (Access and Technology Requirements)],</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please answer 'Yes' or 'No' on applicability
+</t>
+  </si>
+  <si>
+    <t>Sch A 2aii</t>
+  </si>
+  <si>
+    <t>EY will perform the Onboarding Services to [insert general high-level objective]. Onboarding Services will consist of [insert general high-level description of services].</t>
+  </si>
+  <si>
+    <t>Onboarding Services - general high-level objective
+Onboarding Services - general high-level description of services</t>
+  </si>
+  <si>
+    <t>Please fill the Onboarding objective and services</t>
+  </si>
+  <si>
+    <t>Sch A 3</t>
+  </si>
+  <si>
+    <t>[NOTE TO DRAFT: Use the following if the Services involve assisting the Client in drafting its conclusions, including its accounting policy manual, as appropriate.] EY will assist Client in documenting its conclusions reached or positions taken on accounting and reporting matters, including the accounting policies Client has selected.</t>
+  </si>
+  <si>
+    <t>Scope - drafting conclusions, including accounting policy manual</t>
+  </si>
+  <si>
     <t>Sch A 5a3</t>
   </si>
   <si>
-    <t>Parent</t>
-  </si>
-  <si>
-    <t>Description of Services</t>
-  </si>
-  <si>
-    <t>Sch_A</t>
+    <t>iii.	Secure Workplace [NOTE TO DRAFT:  Add if EY is providing services from secure bays, as they will drive EY costs.  Be clear where secure bays are being used and which services the secure bays support (to manage costs and scope).] 
+Services in [location(s)] will be conducted out of a Secure Workplace.  Service locations may not be changed without the express written consent of Client.</t>
+  </si>
+  <si>
+    <t>EY is providing services from secure bays, as they will drive EY costs
+location(s)</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please provide location(s)</t>
+  </si>
+  <si>
+    <t>Sch A 5b1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i.	Client shall provide the following environment(s): {Specify the development, testing, integration, implementation and other environments to be provided by Client}. </t>
+  </si>
+  <si>
+    <t>Scope - IT implementation / Operation
+Specify the development, testing, integration, implementation and other environments to be provided by Client</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please answer the second point</t>
+  </si>
+  <si>
+    <t>Sch A 5b6</t>
+  </si>
+  <si>
+    <t>vi.	Client is responsible for any security features associated with the [Implemented/Integrated Software]. [EY will deliver the **IMPL_SOFTWARE** and Deliverables without the implementation of security, and will not be responsible for any delay or increase in expense resulting from the inclusion of security functionality.]</t>
+  </si>
+  <si>
+    <t>Scope - IT implementation / Operation
+Implemented/Integrated Software</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please update the second point</t>
+  </si>
+  <si>
+    <t>IMPL_SOFTWARE, _DESC</t>
+  </si>
+  <si>
+    <t>Sch A 5b7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vii.	Client is responsible for the results of using the **IMPL_SOFTWARE** Software and Deliverables and/or Outputs in its business operations. Client is also responsible for independent verification and testing of such results prior to using them in its business.
+</t>
+  </si>
+  <si>
+    <t>Scope - IT implementation 
+Implemented/Software</t>
   </si>
   <si>
     <t>Sch_B</t>
   </si>
   <si>
-    <t>MANAGED_SVC_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>ONBOARDING_SVC_DESCRIPTION</t>
-  </si>
-  <si>
-    <t>Sch A1bi</t>
-  </si>
-  <si>
-    <t>_ADD1, ADDITIONAL_SVC, _ADD2</t>
-  </si>
-  <si>
-    <t>**ONBOARDING_SVC_DESCRIPTION** as described in Section 1.f</t>
-  </si>
-  <si>
-    <t>Sch A1bii</t>
-  </si>
-  <si>
-    <t>**MANAGED_SVC_DESCRIPTION** as described in Section 3</t>
-  </si>
-  <si>
-    <t>**ADDITIONAL_SVC** Services as described in Section 4</t>
-  </si>
-  <si>
-    <t>Sch A1biii</t>
-  </si>
-  <si>
-    <t>b.	[NOTE TO DRAFT: Include language in brackets if financial accounting and reporting services will be provided] The Services support Client’s business operations and are advisory in nature. EY will not render an assurance report or opinion under this SOW, nor will the Services constitute an audit, review, examination, or other form of assurance as those terms are defined by [Insert the International Auditing and Assurance Standards Board (IAASB) or relevant local standards]. *[Accordingly, EY will not express any form of assurance on accounting matters, financial statements, any financial or other information or internal controls as part of the Services.]* None of the Services or any reports will constitute any legal opinion or advice. EY will not conduct a review to detect fraud or illegal acts.</t>
-  </si>
-  <si>
-    <t>EY will make the Transfer Assistance Services available for up to [(x)] additional months after the effective date of expiration or termination.</t>
+    <t xml:space="preserve">*****B_Schedule***** </t>
+  </si>
+  <si>
+    <t>Service Level Methodology -                                                                                                                                                                                       KPI/SLA driven performance management mechanism, with or without an impact on the fees</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please update schedulle on Service Level Methodology in the SOW template</t>
+  </si>
+  <si>
+    <t>If 'No', delete the entire schedule on Service Level Methodology, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>Sch_D</t>
+  </si>
+  <si>
+    <t>*****D_Schedule*****</t>
+  </si>
+  <si>
+    <t>Governance and Change Control - governance of the Managed Services, roles and responsibilities of both Parties, escalations and maintaining the schedule, type, content, and frequency of the governance meetings
+- Change control procedure and change request template</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please update schedulle on Governance and Change Control in the SOW template</t>
+  </si>
+  <si>
+    <t>If 'No', delete the entire schedule on Governance and Change Control, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>Sch E</t>
+  </si>
+  <si>
+    <t>*****E_Schedule*****</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Access and Technology Requirements - access and technology requirements, i.e., 1.	Network Requirements, 2.	User Access Requirements, 3.	Administrative Access, 4.	Help Desk Access Requirements</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please update schedulle on Access and Technology Requirements in the SOW template</t>
+  </si>
+  <si>
+    <t>If 'No', delete the entire schedule on Access and Technology Requirements, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>Sch_F</t>
+  </si>
+  <si>
+    <t>*****F_Schedule*****</t>
+  </si>
+  <si>
+    <t>Disaster Recovery Plan - access and technology requirements, i.e., 1.	Network Requirements, 2.	User Access Requirements, 3.	Administrative Access, 4.	Help Desk Access Requirements</t>
+  </si>
+  <si>
+    <t>Please answer 'Yes' or 'No' on applicability
+If Yes, Please update schedulle on Disaster Recovery Plan in the SOW template</t>
+  </si>
+  <si>
+    <t>If 'No', delete the entire schedule on Disaster Recovery Plan, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>tableA</t>
+  </si>
+  <si>
+    <t>Client or **CLIENT_FULL_LEGAL_NAME**</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Please update client name from above</t>
+  </si>
+  <si>
+    <t>The twelve (12) month period beginning on the **COMMENCEMENT_DATE** and ending on the first anniversary thereof, and each consecutive twelve (12) month period during the Term of this SOW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract Year </t>
+  </si>
+  <si>
+    <t xml:space="preserve">As defined in Section 6.bb of the SOW.  [NOTE TO DRAFT: Add to definition list if the referenced optional clause is added to the SOW.]  </t>
+  </si>
+  <si>
+    <t>Client-Environment EY Tool</t>
+  </si>
+  <si>
+    <t>Please delete the respective row if 6bb is 'No'</t>
+  </si>
+  <si>
+    <t>A quantity, stated as a number of percentage points that is specified for a given Critical Service Level. The total of all Allocation of Pool Percentages shall not exceed the Pool Percentage Available for Allocation and the quantity of percentage points specified for any Critical Service Level shall not exceed the Maximum SLA Allocation Percentage.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t>Allocation of Pool Percentage</t>
+  </si>
+  <si>
+    <t>Those Service Levels for which a Service Level Credit may be payable. Critical Service Levels are identified in Attachment B-1 (Service Level Matrix). [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Critical Service Level</t>
+  </si>
+  <si>
+    <t>A Service Level Default of a Critical Service Level.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Critical Service Level Default,</t>
+  </si>
+  <si>
+    <t>The methodology used to determine the potential elimination of a Service Level Credit, as described in Section 5 of Schedule B (Service Level Methodology).</t>
+  </si>
+  <si>
+    <t>Earnback</t>
+  </si>
+  <si>
+    <t>Those Service Levels for which no Service Level Credit is payable, but which are meaningful to Client’s business.  Key Measurements are identified in Attachment B-1 (Service Level Metrics).  [NOTE TO DRAFT:  Delete or modify, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Key Measurement, </t>
+  </si>
+  <si>
+    <t>[Twenty-five (25)] percentage points, which would represent [twenty-five percent (25%)] of the At Risk Amount.</t>
+  </si>
+  <si>
+    <t>Maximum SLA Allocation Percentage</t>
+  </si>
+  <si>
+    <t>The time during, or frequency by, which a Service Level shall be measured. The Measurement Window will exclude scheduled maintenance and emergency maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> , Measurement Window,</t>
+  </si>
+  <si>
+    <t>The total {defined term for the EY recurring charges for the Managed Services (per Schedule C)} invoiced by EY in any month for the Managed Services provided to Client, excluding (a) charges for Onboarding Services; (b) taxes, (c) expenses, and (d) one-time charges for Additional Services.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Monthly SLA-Eligible Charges  ,</t>
+  </si>
+  <si>
+    <t>One hundred percentage points (100), which represents one hundred percent (100%) of the At Risk Amount.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pool Percentage Available for Allocation,</t>
+  </si>
+  <si>
+    <t>As defined in Section 1.b of Schedule B (Service Level Methodology).  [Service Levels consist of Critical Service Levels and Key Measurements.]  [NOTE TO DRAFT:  Delete second sentence, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Service Level</t>
+  </si>
+  <si>
+    <t>A credit applied against the Charge as a result of a Service Level Default with respect to a Critical Service level, which credit is specified in Schedule B (Service Level Methodology).  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
+  </si>
+  <si>
+    <t>, Service Level Credit,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EY’s performance for a particular Service Level fails to meet the applicable Service Level (as calculated in accordance with Attachment B-1 (Service Level Metrics)) during the applicable Measurement Window.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Service Level Default,</t>
+  </si>
+  <si>
+    <t>The period, reflected in months, following the [applicable Go-Live Date] for a Service Level, which period is specified in Attachment B-1 (Service Level Matrix).  [NOTE TO DRAFT:  If there is not a Service Level Stabilization Period, delete.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Service Level Stabilization Period, </t>
+  </si>
+  <si>
+    <t>The ** GO_LIVE_DATE**, or as otherwise specified in Attachment B-1 (Service Level Matrix), in the column labeled “Service Level Start Date”.</t>
+  </si>
+  <si>
+    <t>Service Level Start Date</t>
+  </si>
+  <si>
+    <t>Please delete the respective row if Sch B is 'No, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>A Deliverable that is either: (i) a testable configuration made by EY to software, such as a process workflow, or (ii) a software component developed by EY, such as an interface or report format.  [NOTE TO DRAFT: Delete, unless Functional Deliverables are in-scope and applicable.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functional Deliverable, </t>
+  </si>
+  <si>
+    <t>A reproducible condition in a Functional Deliverable that prevents the Functional Deliverable from performing the functions in accordance with the Approved Design such that the Functional Deliverable does not operate or cannot be used in a production environment. [NOTE TO DRAFT: Delete, unless Functional Deliverables are in-scope and applicable.]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nonconformity </t>
+  </si>
+  <si>
+    <t>Please delete the respective row if #6k  is 'No, if Yes, do nothing</t>
+  </si>
+  <si>
+    <t>As defined in Section 1.a of Schedule F (DR Plan).</t>
+  </si>
+  <si>
+    <t>DR Plan</t>
+  </si>
+  <si>
+    <t>Please delete the respective row if Sch F is 'No'</t>
+  </si>
+  <si>
+    <t>As defined in Section 4 of Schedule D (Governance and Change Control).</t>
+  </si>
+  <si>
+    <t>Dispute</t>
+  </si>
+  <si>
+    <t>Please delete the respective row if Sch D is 'No'</t>
+  </si>
+  <si>
+    <t>Client **CLIENT_FULL_LEGAL_NAME** Procedures</t>
+  </si>
+  <si>
+    <t>CLIENT AFFILIATES</t>
+  </si>
+  <si>
+    <t>Ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Affiliate Entity Name </t>
+  </si>
+  <si>
+    <t>Registered Address</t>
+  </si>
+  <si>
+    <t>INSERT FULL LEGAL FIRM NAME</t>
+  </si>
+  <si>
+    <t>OR INSERT as appliable</t>
+  </si>
+  <si>
+    <t>BACKUP</t>
+  </si>
+  <si>
+    <t>Sch_A_1c</t>
   </si>
   <si>
     <t>[NOTE TO DRAFT: Include any limitations of the scope that impact the Onboarding and/or Managed Services.] [Alternative 1: The scope of Services is limited to the following {lines of business, functions, in scope technology}: OR Alternative 2: The scope of Services will not include the following:]</t>
+  </si>
+  <si>
+    <t>[NOTE TO DRAFT: Include any limitations of the scope that impact the Onboarding and/or Managed Services.] [Alternative 1: The scope of Services is limited to the following {lines of business, functions, in scope technology}, Alternative 2: The scope of Services will not include the following:</t>
   </si>
   <si>
     <t>Option 1: The scope of Services is limited to the following {lines of business, functions, in scope technology}.
@@ -650,106 +921,25 @@
     <t>Sch A 1ci</t>
   </si>
   <si>
+    <t>i.        [Insert First scope limitations]</t>
+  </si>
+  <si>
+    <t>Fill the scope limitation</t>
+  </si>
+  <si>
+    <t>Sch_A_1c-2</t>
+  </si>
+  <si>
     <t>Sch A 1cii</t>
   </si>
   <si>
+    <t>i.        [Insert Second scope limitations]</t>
+  </si>
+  <si>
     <t>Sch A 1ciii</t>
   </si>
   <si>
-    <r>
-      <t>i.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">        </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>[Insert First scope limitations]</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>i.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">        </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>[Insert Second scope limitations]</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>i.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">        </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>[Insert Third scope limitations];</t>
-    </r>
-  </si>
-  <si>
-    <t>Fill the scope limitation</t>
-  </si>
-  <si>
-    <t>Sch_A_1c</t>
-  </si>
-  <si>
-    <t>Sch_A_1c-2</t>
-  </si>
-  <si>
-    <t>Sch A 2ai</t>
-  </si>
-  <si>
-    <t>Sch A 2aii</t>
-  </si>
-  <si>
-    <t>Beginning on the Commencement Date [and after Client has completed the necessary technology development activities as described in Schedule E (Access and Technology Requirements)],</t>
-  </si>
-  <si>
-    <t>EY will perform the Onboarding Services to [insert general high-level objective]. Onboarding Services will consist of [insert general high-level description of services].</t>
-  </si>
-  <si>
-    <t>[and after Client has completed the necessary technology development activities as described in Schedule E (Access and Technology Requirements)],</t>
-  </si>
-  <si>
-    <t>Please fill the Onboarding objective and services</t>
+    <t>i.        [Insert Third scope limitations];</t>
   </si>
   <si>
     <t>Sch A 5b2</t>
@@ -773,311 +963,26 @@
     <t>iv.	All hardware and software provided by the Client, including the **IMPL_SOFTWARE**, will perform in accordance with their respective specifications (but EY will not be responsible for any failure of any thereof).</t>
   </si>
   <si>
-    <t xml:space="preserve">vii.	Client is responsible for the results of using the **IMPL_SOFTWARE** Software and Deliverables and/or Outputs in its business operations. Client is also responsible for independent verification and testing of such results prior to using them in its business.
-</t>
-  </si>
-  <si>
-    <t>*****A_Schedule*****</t>
-  </si>
-  <si>
-    <t>Client or **CLIENT_FULL_LEGAL_NAME**</t>
-  </si>
-  <si>
-    <t>The twelve (12) month period beginning on the **COMMENCEMENT_DATE** and ending on the first anniversary thereof, and each consecutive twelve (12) month period during the Term of this SOW.</t>
-  </si>
-  <si>
-    <t>As defined in Section 1.a of Schedule F (DR Plan).</t>
-  </si>
-  <si>
-    <t>Sch_F</t>
-  </si>
-  <si>
-    <t>Allocation of Pool Percentage</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Critical Service Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Critical Service Level Default,</t>
-  </si>
-  <si>
-    <t>Earnback</t>
-  </si>
-  <si>
-    <t>Those Service Levels for which no Service Level Credit is payable, but which are meaningful to Client’s business.  Key Measurements are identified in Attachment B-1 (Service Level Metrics).  [NOTE TO DRAFT:  Delete or modify, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t>A Service Level Default of a Critical Service Level.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t>Those Service Levels for which a Service Level Credit may be payable. Critical Service Levels are identified in Attachment B-1 (Service Level Matrix). [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t>A quantity, stated as a number of percentage points that is specified for a given Critical Service Level. The total of all Allocation of Pool Percentages shall not exceed the Pool Percentage Available for Allocation and the quantity of percentage points specified for any Critical Service Level shall not exceed the Maximum SLA Allocation Percentage.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Key Measurement, </t>
-  </si>
-  <si>
-    <t>Maximum SLA Allocation Percentage</t>
-  </si>
-  <si>
-    <t>The time during, or frequency by, which a Service Level shall be measured. The Measurement Window will exclude scheduled maintenance and emergency maintenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> , Measurement Window,</t>
-  </si>
-  <si>
-    <t>The total {defined term for the EY recurring charges for the Managed Services (per Schedule C)} invoiced by EY in any month for the Managed Services provided to Client, excluding (a) charges for Onboarding Services; (b) taxes, (c) expenses, and (d) one-time charges for Additional Services.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Monthly SLA-Eligible Charges  ,</t>
-  </si>
-  <si>
-    <t>One hundred percentage points (100), which represents one hundred percent (100%) of the At Risk Amount.  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Pool Percentage Available for Allocation,</t>
-  </si>
-  <si>
-    <t>As defined in Section 1.b of Schedule B (Service Level Methodology).  [Service Levels consist of Critical Service Levels and Key Measurements.]  [NOTE TO DRAFT:  Delete second sentence, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Service Level</t>
-  </si>
-  <si>
-    <t>A credit applied against the Charge as a result of a Service Level Default with respect to a Critical Service level, which credit is specified in Schedule B (Service Level Methodology).  [NOTE TO DRAFT:  Delete, unless Service Level Credits will apply.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EY’s performance for a particular Service Level fails to meet the applicable Service Level (as calculated in accordance with Attachment B-1 (Service Level Metrics)) during the applicable Measurement Window.  </t>
-  </si>
-  <si>
-    <t>, Service Level Credit,</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Service Level Default,</t>
-  </si>
-  <si>
-    <t>The period, reflected in months, following the [applicable Go-Live Date] for a Service Level, which period is specified in Attachment B-1 (Service Level Matrix).  [NOTE TO DRAFT:  If there is not a Service Level Stabilization Period, delete.]</t>
-  </si>
-  <si>
-    <t>Service Level Start Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Service Level Stabilization Period, </t>
-  </si>
-  <si>
-    <t>The ** GO_LIVE_DATE**, or as otherwise specified in Attachment B-1 (Service Level Matrix), in the column labeled “Service Level Start Date”.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contract Year </t>
-  </si>
-  <si>
-    <t>A Deliverable that is either: (i) a testable configuration made by EY to software, such as a process workflow, or (ii) a software component developed by EY, such as an interface or report format.  [NOTE TO DRAFT: Delete, unless Functional Deliverables are in-scope and applicable.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Functional Deliverable, </t>
-  </si>
-  <si>
-    <t>A reproducible condition in a Functional Deliverable that prevents the Functional Deliverable from performing the functions in accordance with the Approved Design such that the Functional Deliverable does not operate or cannot be used in a production environment. [NOTE TO DRAFT: Delete, unless Functional Deliverables are in-scope and applicable.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nonconformity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">As defined in Section 6.bb of the SOW.  [NOTE TO DRAFT: Add to definition list if the referenced optional clause is added to the SOW.]  </t>
-  </si>
-  <si>
-    <t>As defined in Section 4 of Schedule D (Governance and Change Control).</t>
-  </si>
-  <si>
-    <t>Sch_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">*****B_Schedule***** </t>
-  </si>
-  <si>
-    <t>Service Level Methodology -                                                                                                                                                                                       KPI/SLA driven performance management mechanism, with or without an impact on the fees</t>
-  </si>
-  <si>
-    <t>*****D_Schedule*****</t>
-  </si>
-  <si>
-    <t>Governance and Change Control - governance of the Managed Services, roles and responsibilities of both Parties, escalations and maintaining the schedule, type, content, and frequency of the governance meetings
-- Change control procedure and change request template</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Access and Technology Requirements - access and technology requirements, i.e., 1.	Network Requirements, 2.	User Access Requirements, 3.	Administrative Access, 4.	Help Desk Access Requirements</t>
-  </si>
-  <si>
-    <t>*****F_Schedule*****</t>
-  </si>
-  <si>
-    <t>Disaster Recovery Plan - access and technology requirements, i.e., 1.	Network Requirements, 2.	User Access Requirements, 3.	Administrative Access, 4.	Help Desk Access Requirements</t>
-  </si>
-  <si>
-    <t>tableA</t>
-  </si>
-  <si>
-    <t>The Services under this SOW shall begin as of **COMMENCEMENT_DATE** (the “Commencement Date”) and end on the date that is  [XX] months after the Go-Live Date (the “Term”).   [NOTE TO DRAFT:  A typical structure might provide for a defined number of months for the Managed Services in relation to the Go-Live Date (or the last of the Go-Live Dates if there is more than one), so that here is a single, coordinated end of the Term for the Managed Services.]</t>
-  </si>
-  <si>
-    <t>The methodology used to determine the potential elimination of a Service Level Credit, as described in Section 5 of Schedule B (Service Level Methodology).</t>
-  </si>
-  <si>
-    <t>[Twenty-five (25)] percentage points, which would represent [twenty-five percent (25%)] of the At Risk Amount.</t>
-  </si>
-  <si>
-    <t>[NOTE TO DRAFT: Include any limitations of the scope that impact the Onboarding and/or Managed Services.] [Alternative 1: The scope of Services is limited to the following {lines of business, functions, in scope technology}, Alternative 2: The scope of Services will not include the following:</t>
-  </si>
-  <si>
-    <t>BACKUP</t>
-  </si>
-  <si>
-    <t>vi.	Client is responsible for any security features associated with the [Implemented/Integrated Software]. [EY will deliver the **IMPL_SOFTWARE** and Deliverables without the implementation of security, and will not be responsible for any delay or increase in expense resulting from the inclusion of security functionality.]</t>
-  </si>
-  <si>
-    <t>IMPL_SOFTWARE, _DESC</t>
-  </si>
-  <si>
-    <t>Please fill as per Summary Text</t>
-  </si>
-  <si>
-    <t>Please select 'No' if not applicable</t>
-  </si>
-  <si>
-    <t>Please fill as per Summary Text, Maximum of 2 to 3 words</t>
-  </si>
-  <si>
-    <t>Please fill as per Summary Text, Maximum of 2 to 3 lines</t>
-  </si>
-  <si>
-    <t>Please mention 'NA' if not applicable, otherwise Please fill as per Summary Text</t>
-  </si>
-  <si>
-    <t>Please mention the applicable  jurisdictional securities laws, e.g., UAE security laws</t>
-  </si>
-  <si>
-    <t>Please select one option from Summary Text</t>
-  </si>
-  <si>
-    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
-Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO, modify if required
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summary Text - 1st point is mandatory, Please select 'Yes' or 'No' on the 2nd point </t>
-  </si>
-  <si>
-    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text
-Consult with Region/local PPD, Region FAAS Quality Leader, MSOC and GCO if 2nd point is applicable</t>
-  </si>
-  <si>
-    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text
-Please update 3rd point, if applicable</t>
-  </si>
-  <si>
-    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
-Please update red text in 2nd point, if applicable</t>
-  </si>
-  <si>
-    <t>Please update commencement date from above</t>
-  </si>
-  <si>
-    <t>Please update '90' days if required
-Please update ## if Applicable. If not, say 'NA'</t>
-  </si>
-  <si>
-    <t>Please update '60' days if required</t>
-  </si>
-  <si>
-    <t>Please update x</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No'</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No'
-If 'yes', Please update x</t>
-  </si>
-  <si>
-    <t>Please provide the full name</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please answer 'Yes' or 'No' on applicability
-</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please provide location(s)</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please answer the second point</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please update the second point</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please update schedulle on Service Level Methodology in the SOW template</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please update schedulle on Governance and Change Control in the SOW template</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please update schedulle on Access and Technology Requirements in the SOW template</t>
-  </si>
-  <si>
-    <t>Please answer 'Yes' or 'No' on applicability
-If Yes, Please update schedulle on Disaster Recovery Plan in the SOW template</t>
-  </si>
-  <si>
-    <t>Please update client name from above</t>
-  </si>
-  <si>
-    <t>Please delete the respective row if 6bb is 'No'</t>
-  </si>
-  <si>
-    <t>Please delete the respective row if Sch B is 'No, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>Please delete the respective row if #6k  is 'No, if Yes, do nothing</t>
-  </si>
-  <si>
-    <t>Please delete the respective row if Sch F is 'No'</t>
-  </si>
-  <si>
-    <t>Please delete the respective row if Sch D is 'No'</t>
-  </si>
-  <si>
-    <t>Please select 'Yes' or 'No' based on the applicability as per Summary Text, 1st point
-Please update text in 2nd point, if applicable</t>
-  </si>
-  <si>
-    <t>f.	EY will conduct the Services under this SOW pursuant to Client’s documented policies and procedures (“Client **CLIENT_FULL_LEGAL_NAME** Procedures”), which as of the Go Live Date is “[Insert Name of Procedures]”, dated **GO_LIVE_DATE** .   Any changes in Client **CLIENT_FULL_LEGAL_NAME** Procedures requested or initiated by Client during the Term will be implemented in accordance with the Change Control Procedures.</t>
-  </si>
-  <si>
-    <t>Client **CLIENT_FULL_LEGAL_NAME** Procedures</t>
-  </si>
-  <si>
-    <t>*****E_Schedule*****</t>
+    <t>All yellow highlighted text needs to be either updated or deleted</t>
+  </si>
+  <si>
+    <t>All text enclosed in [ ] need to be either updated or deleted</t>
+  </si>
+  <si>
+    <t>All text enclosed in [ ] and starting with "NOTE TO DRAFT" need to be deleted</t>
+  </si>
+  <si>
+    <t>All text enclosed in [ ] and not starting with "NOTE TO DRAFT" need to be updated or deleted</t>
+  </si>
+  <si>
+    <t>All text highlighted in blue need not be touched unless specifically mentioned in the clause wise rules</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1086,22 +991,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1131,12 +1023,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1272,7 +1158,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1289,7 +1175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1304,12 +1190,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1339,12 +1225,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="10"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1680,8 +1566,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265DBB42-7CE0-445D-BF3B-D3E1CB2564FA}">
-  <dimension ref="B2:J96"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:K96"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -1692,10 +1578,11 @@
     <col min="6" max="6" width="17.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="73.1796875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="10" width="45" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.1796875" style="1"/>
+    <col min="11" max="11" width="9.1796875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1718,200 +1605,230 @@
         <v>6</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>145</v>
+        <v>7</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" s="11">
         <v>1</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>146</v>
+        <v>12</v>
       </c>
       <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" s="11">
         <v>2</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
-        <v>147</v>
+        <v>14</v>
       </c>
       <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B5" s="11">
         <v>3</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>148</v>
+        <v>16</v>
       </c>
       <c r="J5" s="4"/>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B6" s="11">
         <v>4</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
-        <v>262</v>
+        <v>18</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>5</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="4" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4" t="s">
-        <v>149</v>
+        <v>20</v>
       </c>
       <c r="J7" s="4"/>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B8" s="11">
         <v>6</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="4" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="J8" s="4"/>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B9" s="11">
         <v>7</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="4" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4" t="s">
-        <v>151</v>
+        <v>25</v>
       </c>
       <c r="J9" s="4"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B10" s="11">
         <v>8</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="4" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
-        <v>152</v>
+        <v>28</v>
       </c>
       <c r="J10" s="4"/>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" s="11">
         <v>9</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="4" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>153</v>
+        <v>31</v>
       </c>
       <c r="J11" s="4"/>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>10</v>
       </c>
@@ -1919,20 +1836,23 @@
         <v>1</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="4" t="s">
-        <v>263</v>
+        <v>34</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-    </row>
-    <row r="13" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="11">
         <v>11</v>
       </c>
@@ -1940,20 +1860,23 @@
         <v>1</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
-        <v>264</v>
+        <v>37</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="D14" s="4"/>
@@ -1964,53 +1887,59 @@
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B15" s="11">
         <v>12</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
-        <v>264</v>
+        <v>37</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>172</v>
+        <v>41</v>
       </c>
       <c r="J15" s="4"/>
-    </row>
-    <row r="16" spans="2:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="11">
         <v>13</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>154</v>
+        <v>43</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
-        <v>264</v>
+        <v>37</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>171</v>
+        <v>45</v>
       </c>
       <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="4"/>
@@ -2021,30 +1950,33 @@
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
     </row>
-    <row r="18" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>14</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
-        <v>265</v>
+        <v>49</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>174</v>
+        <v>50</v>
       </c>
       <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="11">
         <v>15</v>
       </c>
@@ -2052,683 +1984,779 @@
         <v>5</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
-        <v>267</v>
+        <v>53</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="11">
         <v>16</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>17</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>180</v>
+        <v>59</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="11">
         <v>18</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
-        <v>272</v>
+        <v>64</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
-    </row>
-    <row r="23" spans="2:10" ht="116" x14ac:dyDescent="0.35">
+      <c r="K22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="116" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="11">
         <v>19</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
-        <v>296</v>
+        <v>68</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
-    </row>
-    <row r="24" spans="2:10" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="159.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="11">
         <v>20</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>155</v>
+        <v>70</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
-        <v>269</v>
+        <v>72</v>
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
-    </row>
-    <row r="25" spans="2:10" ht="149.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="149.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="11">
         <v>21</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>266</v>
+        <v>75</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
-        <v>261</v>
+        <v>11</v>
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
-    </row>
-    <row r="26" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="11">
         <v>22</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
-    </row>
-    <row r="27" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="11">
         <v>23</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>157</v>
+        <v>80</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="4" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
       <c r="J27" s="4"/>
-    </row>
-    <row r="28" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="11">
         <v>24</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
-    </row>
-    <row r="29" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="11">
         <v>25</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>57</v>
+        <v>87</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
-    </row>
-    <row r="30" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="11">
         <v>26</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="4" t="s">
-        <v>273</v>
+        <v>91</v>
       </c>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12"/>
-    </row>
-    <row r="31" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="11">
         <v>27</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="4" t="s">
-        <v>270</v>
+        <v>95</v>
       </c>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
       <c r="J31" s="12"/>
-    </row>
-    <row r="32" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="11">
         <v>28</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>158</v>
+        <v>97</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="F32" s="12"/>
       <c r="G32" s="4" t="s">
-        <v>269</v>
+        <v>72</v>
       </c>
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
-    </row>
-    <row r="33" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="11">
         <v>29</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>68</v>
+        <v>101</v>
       </c>
       <c r="F33" s="12"/>
       <c r="G33" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
-    </row>
-    <row r="34" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="11">
         <v>30</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>71</v>
+        <v>104</v>
       </c>
       <c r="F34" s="12"/>
       <c r="G34" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
-    </row>
-    <row r="35" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="11">
         <v>31</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="F35" s="12"/>
       <c r="G35" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
-    </row>
-    <row r="36" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="11">
         <v>32</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="F36" s="12"/>
       <c r="G36" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
-    </row>
-    <row r="37" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="11">
         <v>33</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4" t="s">
-        <v>271</v>
+        <v>114</v>
       </c>
       <c r="H37" s="4"/>
       <c r="I37" s="4" t="s">
-        <v>159</v>
+        <v>115</v>
       </c>
       <c r="J37" s="4"/>
-    </row>
-    <row r="38" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="11">
         <v>34</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
-    </row>
-    <row r="39" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="11">
         <v>35</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4" t="s">
-        <v>268</v>
+        <v>57</v>
       </c>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
-    </row>
-    <row r="40" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="11">
         <v>36</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>254</v>
+        <v>123</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>274</v>
+        <v>126</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-    </row>
-    <row r="41" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="11">
         <v>37</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
-    </row>
-    <row r="42" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="11">
         <v>38</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4" t="s">
-        <v>275</v>
+        <v>134</v>
       </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
-    </row>
-    <row r="43" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="11">
         <v>39</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4" t="s">
-        <v>276</v>
+        <v>138</v>
       </c>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
-    </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B44" s="11">
         <v>40</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>99</v>
+        <v>139</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4" t="s">
-        <v>277</v>
+        <v>142</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
-    </row>
-    <row r="45" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="11">
         <v>41</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>99</v>
+        <v>139</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>101</v>
+        <v>143</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>102</v>
+        <v>144</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4" t="s">
-        <v>278</v>
+        <v>145</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
       <c r="J45" s="4"/>
-    </row>
-    <row r="46" spans="2:10" ht="125" x14ac:dyDescent="0.35">
+      <c r="K45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:11" ht="125" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="11">
         <v>42</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
       <c r="J46" s="24"/>
-    </row>
-    <row r="47" spans="2:10" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:11" ht="159.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="11">
         <v>43</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>104</v>
+        <v>150</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>105</v>
+        <v>152</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4" t="s">
-        <v>279</v>
+        <v>153</v>
       </c>
       <c r="H47" s="4"/>
       <c r="I47" s="23"/>
       <c r="J47" s="22"/>
-    </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B48" s="11">
         <v>44</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>106</v>
+        <v>154</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>107</v>
+        <v>156</v>
       </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4" t="s">
-        <v>280</v>
+        <v>157</v>
       </c>
       <c r="H48" s="4"/>
       <c r="I48" s="23"/>
       <c r="J48" s="22"/>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B49" s="11">
         <v>45</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>108</v>
+        <v>158</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>109</v>
+        <v>160</v>
       </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4" t="s">
-        <v>280</v>
+        <v>157</v>
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="23"/>
       <c r="J49" s="22"/>
-    </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B50" s="11">
         <v>46</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>207</v>
+        <v>162</v>
       </c>
       <c r="E50" s="20" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4" t="s">
-        <v>281</v>
+        <v>164</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="23"/>
       <c r="J50" s="22"/>
-    </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B51" s="11"/>
       <c r="C51" s="19" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="D51" s="28" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="E51" s="27"/>
       <c r="F51" s="4"/>
@@ -2736,16 +2764,16 @@
       <c r="H51" s="4"/>
       <c r="I51" s="23"/>
       <c r="J51" s="22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B52" s="11"/>
       <c r="C52" s="19" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="D52" s="28" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E52" s="27"/>
       <c r="F52" s="4"/>
@@ -2753,16 +2781,16 @@
       <c r="H52" s="4"/>
       <c r="I52" s="23"/>
       <c r="J52" s="22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B53" s="11"/>
       <c r="C53" s="19" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="D53" s="28" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="E53" s="27"/>
       <c r="F53" s="4"/>
@@ -2770,16 +2798,16 @@
       <c r="H53" s="4"/>
       <c r="I53" s="23"/>
       <c r="J53" s="22" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="58" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="58" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="11"/>
       <c r="C58" s="11" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="D58" s="21" t="s">
-        <v>297</v>
+        <v>172</v>
       </c>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
@@ -2787,173 +2815,194 @@
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="59" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="59" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="11">
         <v>47</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>197</v>
+        <v>174</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4" t="s">
-        <v>282</v>
+        <v>176</v>
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
       <c r="J59" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="60" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="11">
         <v>48</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
       <c r="J60" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="61" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="11">
         <v>49</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>111</v>
+        <v>181</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>112</v>
+        <v>182</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>113</v>
+        <v>183</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4" t="s">
-        <v>281</v>
+        <v>164</v>
       </c>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="62" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="11">
         <v>50</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>114</v>
+        <v>185</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>115</v>
+        <v>186</v>
       </c>
       <c r="F62" s="4"/>
       <c r="G62" s="4" t="s">
-        <v>283</v>
+        <v>187</v>
       </c>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
       <c r="J62" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="63" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="11">
         <v>51</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>116</v>
+        <v>188</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>117</v>
+        <v>189</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>118</v>
+        <v>190</v>
       </c>
       <c r="F63" s="4"/>
       <c r="G63" s="4" t="s">
-        <v>284</v>
+        <v>191</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
       <c r="J63" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="67" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="11">
         <v>52</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>119</v>
+        <v>192</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>259</v>
+        <v>193</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="F67" s="4"/>
       <c r="G67" s="4" t="s">
-        <v>285</v>
+        <v>195</v>
       </c>
       <c r="H67" s="4"/>
       <c r="I67" s="4" t="s">
-        <v>260</v>
+        <v>196</v>
       </c>
       <c r="J67" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="68" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="11">
         <v>53</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>121</v>
+        <v>197</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>122</v>
+        <v>199</v>
       </c>
       <c r="F68" s="4"/>
       <c r="G68" s="4" t="s">
-        <v>281</v>
+        <v>164</v>
       </c>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
       <c r="J68" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="69" spans="2:10" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B69" s="11"/>
       <c r="C69" s="11"/>
       <c r="D69" s="4"/>
@@ -2964,545 +3013,557 @@
       <c r="I69" s="4"/>
       <c r="J69" s="26"/>
     </row>
-    <row r="70" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="11">
         <v>54</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>246</v>
+        <v>201</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>247</v>
+        <v>202</v>
       </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4" t="s">
-        <v>286</v>
+        <v>203</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>123</v>
+        <v>204</v>
       </c>
       <c r="I70" s="4"/>
       <c r="J70" s="4"/>
-    </row>
-    <row r="71" spans="2:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:11" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="11">
         <v>55</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>245</v>
+        <v>205</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>248</v>
+        <v>206</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>249</v>
+        <v>207</v>
       </c>
       <c r="F71" s="4"/>
       <c r="G71" s="4" t="s">
-        <v>287</v>
+        <v>208</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>124</v>
+        <v>209</v>
       </c>
       <c r="I71" s="4"/>
       <c r="J71" s="4"/>
-    </row>
-    <row r="72" spans="2:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:11" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B72" s="11">
         <v>56</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>125</v>
+        <v>210</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>299</v>
+        <v>211</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>250</v>
+        <v>212</v>
       </c>
       <c r="F72" s="4"/>
       <c r="G72" s="4" t="s">
-        <v>288</v>
+        <v>213</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>126</v>
+        <v>214</v>
       </c>
       <c r="I72" s="4"/>
       <c r="J72" s="4"/>
-    </row>
-    <row r="73" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="11">
         <v>57</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>251</v>
+        <v>216</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>252</v>
+        <v>217</v>
       </c>
       <c r="F73" s="4"/>
       <c r="G73" s="4" t="s">
-        <v>289</v>
+        <v>218</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>127</v>
+        <v>219</v>
       </c>
       <c r="I73" s="4"/>
       <c r="J73" s="4"/>
-    </row>
-    <row r="74" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="K73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B74" s="11"/>
       <c r="C74" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>290</v>
+        <v>223</v>
       </c>
       <c r="I74" s="4"/>
       <c r="J74" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="75" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="75" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="11"/>
       <c r="C75" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>274</v>
+        <v>126</v>
       </c>
       <c r="I75" s="4"/>
       <c r="J75" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="76" spans="2:10" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="76" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B76" s="11"/>
       <c r="C76" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>129</v>
+        <v>227</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>291</v>
+        <v>228</v>
       </c>
       <c r="I76" s="4"/>
       <c r="J76" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="77" spans="2:10" ht="37.5" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="77" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="11"/>
       <c r="C77" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D77" s="31" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
       <c r="J77" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="78" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="78" spans="2:11" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C78" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D78" s="31" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
       <c r="J78" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="79" spans="2:10" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="79" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B79" s="11"/>
       <c r="C79" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D79" s="29" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="F79" s="4"/>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
       <c r="J79" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="80" spans="2:10" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="80" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B80" s="11"/>
       <c r="C80" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D80" s="31" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="F80" s="4"/>
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
       <c r="J80" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="81" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="81" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="11"/>
       <c r="C81" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D81" s="31" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="F81" s="4"/>
       <c r="G81" s="4"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
       <c r="J81" s="4" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
     </row>
     <row r="82" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B82" s="11"/>
       <c r="C82" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D82" s="31" t="s">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="F82" s="4"/>
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
       <c r="J82" s="4" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
     </row>
     <row r="83" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B83" s="11"/>
       <c r="C83" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D83" s="31" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="F83" s="4"/>
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
       <c r="J83" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="84" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="84" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="11"/>
       <c r="C84" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D84" s="31" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="F84" s="4"/>
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
       <c r="J84" s="4" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
     </row>
     <row r="85" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B85" s="11"/>
       <c r="C85" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D85" s="31" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="F85" s="4"/>
       <c r="G85" s="4"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
       <c r="J85" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="86" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="86" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="11"/>
       <c r="C86" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D86" s="31" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="F86" s="4"/>
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
       <c r="J86" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="87" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="87" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="11"/>
       <c r="C87" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D87" s="31" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="F87" s="4"/>
       <c r="G87" s="4"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
       <c r="J87" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="88" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="88" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="11"/>
       <c r="C88" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D88" s="31" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="F88" s="4"/>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
       <c r="J88" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="89" spans="2:10" ht="25" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="89" spans="2:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="11"/>
       <c r="C89" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="D89" s="31" t="s">
         <v>253</v>
       </c>
-      <c r="D89" s="31" t="s">
-        <v>234</v>
-      </c>
       <c r="E89" s="4" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="F89" s="4"/>
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
       <c r="J89" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="90" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="90" spans="2:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="11"/>
       <c r="C90" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>235</v>
+        <v>256</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>292</v>
+        <v>257</v>
       </c>
       <c r="I90" s="4"/>
       <c r="J90" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="91" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="91" spans="2:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="11"/>
       <c r="C91" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="F91" s="4"/>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
       <c r="J91" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="92" spans="2:10" ht="29" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="92" spans="2:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="11"/>
       <c r="C92" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>293</v>
+        <v>262</v>
       </c>
       <c r="I92" s="4"/>
       <c r="J92" s="4" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
     </row>
     <row r="93" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B93" s="11"/>
       <c r="C93" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>210</v>
+        <v>263</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>130</v>
+        <v>264</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>294</v>
+        <v>265</v>
       </c>
       <c r="I93" s="4"/>
       <c r="J93" s="4" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="94" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B94" s="11"/>
       <c r="C94" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>131</v>
+        <v>267</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="I94" s="4"/>
       <c r="J94" s="4" t="s">
-        <v>245</v>
+        <v>205</v>
       </c>
     </row>
     <row r="95" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B95" s="11"/>
       <c r="C95" s="11" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>298</v>
+        <v>269</v>
       </c>
       <c r="E95" s="4"/>
       <c r="F95" s="4"/>
@@ -3523,15 +3584,14 @@
       <c r="J96" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:H92" xr:uid="{265DBB42-7CE0-445D-BF3B-D3E1CB2564FA}"/>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <autoFilter ref="B2:H92" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F5AEE25-55E7-432F-AF5D-061A9E120231}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:J21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3542,18 +3602,18 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
-        <v>132</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
-        <v>133</v>
+        <v>271</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>134</v>
+        <v>272</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>135</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.35">
@@ -3561,7 +3621,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>136</v>
+        <v>274</v>
       </c>
       <c r="D4" s="8"/>
     </row>
@@ -3570,7 +3630,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>136</v>
+        <v>274</v>
       </c>
       <c r="D5" s="8"/>
     </row>
@@ -3579,7 +3639,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>136</v>
+        <v>274</v>
       </c>
       <c r="D6" s="8"/>
     </row>
@@ -3588,21 +3648,21 @@
         <v>4</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>136</v>
+        <v>274</v>
       </c>
       <c r="D7" s="8"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C9" s="9" t="s">
-        <v>137</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="10" t="s">
         <v>0</v>
       </c>
@@ -3625,134 +3685,134 @@
         <v>6</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>145</v>
+        <v>7</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" ht="409.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="409.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="11">
         <v>47</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>191</v>
+        <v>277</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>182</v>
+        <v>278</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
-        <v>183</v>
+        <v>280</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="23"/>
       <c r="J15" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="11">
         <v>48</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>184</v>
+        <v>281</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>187</v>
+        <v>282</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="23"/>
       <c r="J16" s="25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="11">
         <v>49</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>185</v>
+        <v>285</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>188</v>
+        <v>286</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="23"/>
       <c r="J17" s="25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>50</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>186</v>
+        <v>287</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>189</v>
+        <v>288</v>
       </c>
       <c r="E18" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="27" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="23"/>
       <c r="J18" s="25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" ht="409.5" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" ht="409.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="11">
         <v>56</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>199</v>
+        <v>289</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>200</v>
+        <v>290</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>201</v>
+        <v>291</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="s">
-        <v>202</v>
+        <v>292</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>203</v>
+        <v>293</v>
       </c>
       <c r="J19" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="87" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="87" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
       <c r="D20" s="4" t="s">
-        <v>204</v>
+        <v>294</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -3760,14 +3820,14 @@
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="D21" s="4" t="s">
-        <v>205</v>
+        <v>295</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -3775,7 +3835,7 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="25" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3784,16 +3844,16 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0189E61E-37D7-4696-83EA-025EC3498A9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B3:L7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:12" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B3" s="15">
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>138</v>
+        <v>296</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
@@ -3805,12 +3865,12 @@
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
     </row>
-    <row r="4" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="4" spans="2:12" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B4" s="15">
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>139</v>
+        <v>297</v>
       </c>
       <c r="D4" s="15"/>
       <c r="E4" s="15"/>
@@ -3822,12 +3882,12 @@
       <c r="K4" s="15"/>
       <c r="L4" s="15"/>
     </row>
-    <row r="5" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:12" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="15">
         <v>3</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>140</v>
+        <v>298</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
@@ -3839,12 +3899,12 @@
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
     </row>
-    <row r="6" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="6" spans="2:12" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B6" s="15">
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>141</v>
+        <v>299</v>
       </c>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
@@ -3856,12 +3916,12 @@
       <c r="K6" s="15"/>
       <c r="L6" s="15"/>
     </row>
-    <row r="7" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="7" spans="2:12" ht="26" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B7" s="15">
         <v>5</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>142</v>
+        <v>300</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
@@ -3875,200 +3935,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100512D8143EBAB4F48A45D02323B7787CD" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="615fc09795e7468283b6f0bb7d04746b">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="63b1587f-e08d-4165-8b7c-8e10ec81d5e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c75373169537aa6399a5b51c659de3c9" ns2:_="">
-    <xsd:import namespace="63b1587f-e08d-4165-8b7c-8e10ec81d5e9"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="63b1587f-e08d-4165-8b7c-8e10ec81d5e9" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F181C95-A625-4FA9-AB3F-4518C4A67DA5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="63b1587f-e08d-4165-8b7c-8e10ec81d5e9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2053D39-4E93-4F4E-A5B5-F28709406B08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1138237B-C0C9-4654-A68E-00C5B91EEAD3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>